<commit_message>
docs: regenerate produits_template.xlsx to include  header
</commit_message>
<xml_diff>
--- a/front-react/public/produits_template.xlsx
+++ b/front-react/public/produits_template.xlsx
@@ -410,7 +410,7 @@
         <v>id_unite</v>
       </c>
       <c r="D1" t="str">
-        <v>unite_code</v>
+        <v>symbole</v>
       </c>
       <c r="E1" t="str">
         <v>unite_name</v>
@@ -486,7 +486,7 @@
         <v/>
       </c>
       <c r="D3" t="str">
-        <v/>
+        <v>BOÎTE</v>
       </c>
       <c r="E3" t="str">
         <v>Boîte</v>

</xml_diff>